<commit_message>
Sample book v14: README and tracker (RCM 2026 photos, MECSR Verified seal)
README and tracker (repository edition, no personal data) for sample book v14. The v14 PDFs and the rebuilt index.html follow in the next commit.
</commit_message>
<xml_diff>
--- a/MECSR_2027_Directory_Content_Tracker.xlsx
+++ b/MECSR_2027_Directory_Content_Tracker.xlsx
@@ -936,7 +936,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>12 Oct 2026 — sample book v13: every QR code taken out of print (listing addresses change when a listing is renamed); pages 5, 78 and 381 rewritten to match. Earlier — 10 Oct 2026 — RCM matrix of 8 Oct applied (Champion Group provisional, Ground Control, Kingdom Centre, Dhamani, Eleva AI); 04 Flat Plan moved to the v12 pagination (every spread starts on a left-hand page); intel sheets 10–12 and a book QA sheet (13) added.</t>
+          <t>13 Oct 2026 — sample book v14: Retail Congress MENA 2026 photographs on the MENA Awards page (66) and the other house ads (67–69), each showcase sponsor's own congress stand on its imagery page (21–31), and stand-ins on the Expert Views (38–54), the leadership messages (6–8) and the Title Partner page (2); the MECSR Verified seal on the 341 listings that carry a photograph and on the 7 Must-Visit pages, explained on p78. Earlier — 12 Oct 2026 — sample book v13: every QR code taken out of print (listing addresses change when a listing is renamed); pages 5, 78 and 381 rewritten to match. Earlier — 10 Oct 2026 — RCM matrix of 8 Oct applied (Champion Group provisional, Ground Control, Kingdom Centre, Dhamani, Eleva AI); 04 Flat Plan moved to the v12 pagination (every spread starts on a left-hand page); intel sheets 10–12 and a book QA sheet (13) added.</t>
         </is>
       </c>
     </row>
@@ -1287,7 +1287,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="32" customHeight="1" s="72">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -2221,7 +2220,6 @@
       <c r="M18" s="80" t="inlineStr"/>
       <c r="N18" s="80" t="inlineStr"/>
     </row>
-    <row r="19"/>
     <row r="20" ht="40" customHeight="1" s="72">
       <c r="B20" s="84" t="inlineStr">
         <is>
@@ -2296,7 +2294,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="32" customHeight="1" s="72">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -4377,7 +4374,6 @@
       <c r="I54" s="80" t="inlineStr"/>
       <c r="J54" s="80" t="inlineStr"/>
     </row>
-    <row r="55"/>
     <row r="56" ht="40" customHeight="1" s="72">
       <c r="B56" s="84" t="inlineStr">
         <is>
@@ -4433,7 +4429,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="32" customHeight="1" s="72">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -5368,7 +5363,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="32" customHeight="1" s="72">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -6021,7 +6015,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="26" customHeight="1" s="72">
       <c r="B23" s="71" t="inlineStr">
         <is>
@@ -6079,7 +6072,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="32" customHeight="1" s="72">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -6459,7 +6451,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="32" customHeight="1" s="72">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -7205,7 +7196,11 @@
       <c r="M6" s="11" t="n"/>
       <c r="N6" s="11" t="n"/>
       <c r="O6" s="11" t="n"/>
-      <c r="P6" s="11" t="n"/>
+      <c r="P6" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: stand-in photo (main hall, Retail Congress MENA 2026) until the title partner supplies artwork.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="26" customHeight="1" s="72">
       <c r="A7" s="8" t="n">
@@ -7421,7 +7416,11 @@
       <c r="M10" s="11" t="n"/>
       <c r="N10" s="11" t="n"/>
       <c r="O10" s="11" t="n"/>
-      <c r="P10" s="11" t="n"/>
+      <c r="P10" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: congress photo below the message; the portrait is still to be supplied.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="26" customHeight="1" s="72">
       <c r="A11" s="8" t="n">
@@ -7475,7 +7474,11 @@
       <c r="M11" s="11" t="n"/>
       <c r="N11" s="11" t="n"/>
       <c r="O11" s="11" t="n"/>
-      <c r="P11" s="11" t="n"/>
+      <c r="P11" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: congress photo below the message; the portrait is still to be supplied.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="26" customHeight="1" s="72">
       <c r="A12" s="8" t="n">
@@ -7529,7 +7532,11 @@
       <c r="M12" s="11" t="n"/>
       <c r="N12" s="11" t="n"/>
       <c r="O12" s="11" t="n"/>
-      <c r="P12" s="11" t="n"/>
+      <c r="P12" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: congress photo below the message; the portrait is still to be supplied.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="26" customHeight="1" s="72">
       <c r="A13" s="8" t="n">
@@ -7907,7 +7914,11 @@
       <c r="M19" s="11" t="n"/>
       <c r="N19" s="11" t="n"/>
       <c r="O19" s="11" t="n"/>
-      <c r="P19" s="11" t="n"/>
+      <c r="P19" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: the sponsor's own stand at Retail Congress MENA 2026 stands in for the imagery brief (right-hand page).</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="26" customHeight="1" s="72">
       <c r="A20" s="8" t="n">
@@ -7961,7 +7972,11 @@
       <c r="M20" s="11" t="n"/>
       <c r="N20" s="11" t="n"/>
       <c r="O20" s="11" t="n"/>
-      <c r="P20" s="11" t="n"/>
+      <c r="P20" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: the sponsor's own stand at Retail Congress MENA 2026 stands in for the imagery brief (right-hand page).</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="26" customHeight="1" s="72">
       <c r="A21" s="8" t="n">
@@ -8015,7 +8030,11 @@
       <c r="M21" s="11" t="n"/>
       <c r="N21" s="11" t="n"/>
       <c r="O21" s="11" t="n"/>
-      <c r="P21" s="11" t="n"/>
+      <c r="P21" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: the sponsor's own stand at Retail Congress MENA 2026 stands in for the imagery brief (right-hand page).</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="26" customHeight="1" s="72">
       <c r="A22" s="8" t="n">
@@ -8069,7 +8088,11 @@
       <c r="M22" s="11" t="n"/>
       <c r="N22" s="11" t="n"/>
       <c r="O22" s="11" t="n"/>
-      <c r="P22" s="11" t="n"/>
+      <c r="P22" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: the sponsor's own stand at Retail Congress MENA 2026 stands in for the imagery brief (right-hand page).</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="26" customHeight="1" s="72">
       <c r="A23" s="8" t="n">
@@ -8123,7 +8146,11 @@
       <c r="M23" s="11" t="n"/>
       <c r="N23" s="11" t="n"/>
       <c r="O23" s="11" t="n"/>
-      <c r="P23" s="11" t="n"/>
+      <c r="P23" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: the sponsor's own stand at Retail Congress MENA 2026 stands in for the imagery brief (right-hand page).</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="26" customHeight="1" s="72">
       <c r="A24" s="8" t="n">
@@ -8177,7 +8204,11 @@
       <c r="M24" s="11" t="n"/>
       <c r="N24" s="11" t="n"/>
       <c r="O24" s="11" t="n"/>
-      <c r="P24" s="11" t="n"/>
+      <c r="P24" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: the sponsor's own stand at Retail Congress MENA 2026 stands in for the imagery brief (right-hand page).</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="26" customHeight="1" s="72">
       <c r="A25" s="8" t="n">
@@ -8393,7 +8424,11 @@
       <c r="M28" s="11" t="n"/>
       <c r="N28" s="11" t="n"/>
       <c r="O28" s="11" t="n"/>
-      <c r="P28" s="11" t="n"/>
+      <c r="P28" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: a congress photo stands in for the author's supporting images; the headshot is still to be supplied.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="26" customHeight="1" s="72">
       <c r="A29" s="8" t="n">
@@ -8447,7 +8482,11 @@
       <c r="M29" s="11" t="n"/>
       <c r="N29" s="11" t="n"/>
       <c r="O29" s="11" t="n"/>
-      <c r="P29" s="11" t="n"/>
+      <c r="P29" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: a congress photo stands in for the author's supporting images; the headshot is still to be supplied.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="26" customHeight="1" s="72">
       <c r="A30" s="8" t="n">
@@ -8501,7 +8540,11 @@
       <c r="M30" s="11" t="n"/>
       <c r="N30" s="11" t="n"/>
       <c r="O30" s="11" t="n"/>
-      <c r="P30" s="11" t="n"/>
+      <c r="P30" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: a congress photo stands in for the author's supporting images; the headshot is still to be supplied.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="26" customHeight="1" s="72">
       <c r="A31" s="8" t="n">
@@ -8555,7 +8598,11 @@
       <c r="M31" s="11" t="n"/>
       <c r="N31" s="11" t="n"/>
       <c r="O31" s="11" t="n"/>
-      <c r="P31" s="11" t="n"/>
+      <c r="P31" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: a congress photo stands in for the author's supporting images; the headshot is still to be supplied.</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="26" customHeight="1" s="72">
       <c r="A32" s="8" t="n">
@@ -8609,7 +8656,11 @@
       <c r="M32" s="11" t="n"/>
       <c r="N32" s="11" t="n"/>
       <c r="O32" s="11" t="n"/>
-      <c r="P32" s="11" t="n"/>
+      <c r="P32" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: a congress photo stands in for the author's supporting images; the headshot is still to be supplied.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="26" customHeight="1" s="72">
       <c r="A33" s="8" t="n">
@@ -8663,7 +8714,11 @@
       <c r="M33" s="11" t="n"/>
       <c r="N33" s="11" t="n"/>
       <c r="O33" s="11" t="n"/>
-      <c r="P33" s="11" t="n"/>
+      <c r="P33" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: a congress photo stands in for the author's supporting images; the headshot is still to be supplied.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="26" customHeight="1" s="72">
       <c r="A34" s="8" t="n">
@@ -8717,7 +8772,11 @@
       <c r="M34" s="11" t="n"/>
       <c r="N34" s="11" t="n"/>
       <c r="O34" s="11" t="n"/>
-      <c r="P34" s="11" t="n"/>
+      <c r="P34" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: a congress photo stands in for the author's supporting images; the headshot is still to be supplied.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="26" customHeight="1" s="72">
       <c r="A35" s="8" t="n">
@@ -8771,7 +8830,11 @@
       <c r="M35" s="11" t="n"/>
       <c r="N35" s="11" t="n"/>
       <c r="O35" s="11" t="n"/>
-      <c r="P35" s="11" t="n"/>
+      <c r="P35" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: a congress photo stands in for the author's supporting images; the headshot is still to be supplied.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="26" customHeight="1" s="72">
       <c r="A36" s="8" t="n">
@@ -8825,7 +8888,11 @@
       <c r="M36" s="11" t="n"/>
       <c r="N36" s="11" t="n"/>
       <c r="O36" s="11" t="n"/>
-      <c r="P36" s="11" t="n"/>
+      <c r="P36" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: a congress photo stands in for the author's supporting images; the headshot is still to be supplied.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="26" customHeight="1" s="72">
       <c r="A37" s="8" t="n">
@@ -9149,7 +9216,11 @@
       <c r="M42" s="11" t="n"/>
       <c r="N42" s="11" t="n"/>
       <c r="O42" s="11" t="n"/>
-      <c r="P42" s="11" t="n"/>
+      <c r="P42" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: designed with MENA Awards 2026 photography (winners on stage).</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="26" customHeight="1" s="72">
       <c r="A43" s="8" t="n">
@@ -9203,7 +9274,11 @@
       <c r="M43" s="11" t="n"/>
       <c r="N43" s="11" t="n"/>
       <c r="O43" s="11" t="n"/>
-      <c r="P43" s="11" t="n"/>
+      <c r="P43" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: designed with Retail Congress MENA 2026 photography.</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="26" customHeight="1" s="72">
       <c r="A44" s="8" t="n">
@@ -9257,7 +9332,11 @@
       <c r="M44" s="11" t="n"/>
       <c r="N44" s="11" t="n"/>
       <c r="O44" s="11" t="n"/>
-      <c r="P44" s="11" t="n"/>
+      <c r="P44" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: designed with Retail Congress MENA 2026 photography.</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="26" customHeight="1" s="72">
       <c r="A45" s="8" t="n">
@@ -9311,7 +9390,11 @@
       <c r="M45" s="11" t="n"/>
       <c r="N45" s="11" t="n"/>
       <c r="O45" s="11" t="n"/>
-      <c r="P45" s="11" t="n"/>
+      <c r="P45" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: designed with Retail Congress MENA 2026 photography.</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="26" customHeight="1" s="72">
       <c r="A46" s="8" t="n">
@@ -9419,7 +9502,11 @@
       <c r="M47" s="11" t="n"/>
       <c r="N47" s="11" t="n"/>
       <c r="O47" s="11" t="n"/>
-      <c r="P47" s="11" t="n"/>
+      <c r="P47" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: MECSR Verified seal beside the centre name.</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="26" customHeight="1" s="72">
       <c r="A48" s="8" t="n">
@@ -9473,7 +9560,11 @@
       <c r="M48" s="11" t="n"/>
       <c r="N48" s="11" t="n"/>
       <c r="O48" s="11" t="n"/>
-      <c r="P48" s="11" t="n"/>
+      <c r="P48" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: MECSR Verified seal beside the centre name.</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="26" customHeight="1" s="72">
       <c r="A49" s="8" t="n">
@@ -9527,7 +9618,11 @@
       <c r="M49" s="11" t="n"/>
       <c r="N49" s="11" t="n"/>
       <c r="O49" s="11" t="n"/>
-      <c r="P49" s="11" t="n"/>
+      <c r="P49" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: MECSR Verified seal beside the centre name.</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="26" customHeight="1" s="72">
       <c r="A50" s="8" t="n">
@@ -9581,7 +9676,11 @@
       <c r="M50" s="11" t="n"/>
       <c r="N50" s="11" t="n"/>
       <c r="O50" s="11" t="n"/>
-      <c r="P50" s="11" t="n"/>
+      <c r="P50" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: MECSR Verified seal beside the centre name.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="26" customHeight="1" s="72">
       <c r="A51" s="8" t="n">
@@ -9635,7 +9734,11 @@
       <c r="M51" s="11" t="n"/>
       <c r="N51" s="11" t="n"/>
       <c r="O51" s="11" t="n"/>
-      <c r="P51" s="11" t="n"/>
+      <c r="P51" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: MECSR Verified seal beside the centre name.</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="26" customHeight="1" s="72">
       <c r="A52" s="8" t="n">
@@ -9689,7 +9792,11 @@
       <c r="M52" s="11" t="n"/>
       <c r="N52" s="11" t="n"/>
       <c r="O52" s="11" t="n"/>
-      <c r="P52" s="11" t="n"/>
+      <c r="P52" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: MECSR Verified seal beside the centre name.</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="26" customHeight="1" s="72">
       <c r="A53" s="8" t="n">
@@ -9743,7 +9850,11 @@
       <c r="M53" s="11" t="n"/>
       <c r="N53" s="11" t="n"/>
       <c r="O53" s="11" t="n"/>
-      <c r="P53" s="11" t="n"/>
+      <c r="P53" s="11" t="inlineStr">
+        <is>
+          <t>v14 sample: MECSR Verified seal beside the centre name.</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="26" customHeight="1" s="72">
       <c r="A54" s="8" t="n">
@@ -9797,7 +9908,11 @@
       <c r="M54" s="11" t="n"/>
       <c r="N54" s="11" t="n"/>
       <c r="O54" s="11" t="n"/>
-      <c r="P54" s="11" t="n"/>
+      <c r="P54" s="11" t="inlineStr">
+        <is>
+          <t>v14: legend for the MECSR Verified seal added on p78.</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="26" customHeight="1" s="72">
       <c r="A55" s="8" t="n">
@@ -11903,7 +12018,11 @@
       <c r="M93" s="11" t="n"/>
       <c r="N93" s="11" t="n"/>
       <c r="O93" s="11" t="n"/>
-      <c r="P93" s="11" t="n"/>
+      <c r="P93" s="11" t="inlineStr">
+        <is>
+          <t>v14: photography note added (RCM 2026 stand-in photos; the seal on sample listings).</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="26" customHeight="1" s="72">
       <c r="A94" s="8" t="n">
@@ -12683,7 +12802,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="32" customHeight="1" s="72">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -13333,7 +13451,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27" ht="32" customHeight="1" s="72">
       <c r="B27" s="71" t="inlineStr">
         <is>
@@ -13398,7 +13515,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="32" customHeight="1" s="72">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -13913,7 +14029,6 @@
       <c r="O13" s="11" t="n"/>
       <c r="P13" s="11" t="n"/>
     </row>
-    <row r="14"/>
     <row r="15" ht="34.05" customHeight="1" s="72">
       <c r="B15" s="71" t="inlineStr">
         <is>
@@ -13987,7 +14102,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="32" customHeight="1" s="72">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -20064,7 +20178,6 @@
       <c r="T67" s="80" t="inlineStr"/>
       <c r="U67" s="80" t="inlineStr"/>
     </row>
-    <row r="68"/>
     <row r="69" ht="40" customHeight="1" s="72">
       <c r="B69" s="84" t="inlineStr">
         <is>
@@ -20193,7 +20306,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="32" customHeight="1" s="72">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -23418,7 +23530,6 @@
       <c r="O49" s="80" t="inlineStr"/>
       <c r="P49" s="80" t="inlineStr"/>
     </row>
-    <row r="50"/>
     <row r="51" ht="40" customHeight="1" s="72">
       <c r="B51" s="84" t="inlineStr">
         <is>

</xml_diff>